<commit_message>
Refresh aircraft facts from the spreadsheet; default to YOW at 50 km
- Regenerate lib/facts.ts from the updated fun-facts workbook: 36 -> 92
  aircraft types, refreshed copy, and alias cleanup for the new rows.
- Default station is now the airport itself, not a Nepean postal code.
- Default radar range 25 -> 50 km; station field placeholder is YOW's
  postal code (K1V 9B4).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/ottawa_aircraft_fun_facts.xlsx
+++ b/data/ottawa_aircraft_fun_facts.xlsx
@@ -469,18 +469,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:I93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="55" customWidth="1" min="7" max="7"/>
-    <col width="55" customWidth="1" min="8" max="8"/>
-    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="58" customWidth="1" min="7" max="7"/>
+    <col width="58" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -530,7 +530,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="60" customHeight="1">
+    <row r="2" ht="62" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>A320</t>
@@ -553,7 +553,7 @@
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t>Air Canada, Air Canada Rouge, WestJet, Sunwing</t>
+          <t>Air Canada, Air Canada Rouge, WestJet</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr">
@@ -577,7 +577,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="60" customHeight="1">
+    <row r="3" ht="62" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
           <t>A321</t>
@@ -624,7 +624,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="60" customHeight="1">
+    <row r="4" ht="62" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>A319</t>
@@ -667,7 +667,7 @@
       </c>
       <c r="I4" s="3" t="inlineStr"/>
     </row>
-    <row r="5" ht="60" customHeight="1">
+    <row r="5" ht="62" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>BCS3</t>
@@ -714,7 +714,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="60" customHeight="1">
+    <row r="6" ht="62" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>B738</t>
@@ -737,7 +737,7 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>WestJet, Sunwing, Air Canada</t>
+          <t>WestJet, Air Canada</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -747,7 +747,7 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>The 737-800 is part of the best-selling "Next Generation" 737 family and remains the backbone of WestJet's entire fleet.</t>
+          <t>The 737-800 is part of the best-selling "Next Generation" 737 family and remains the backbone of WestJet's entire fleet, which absorbed Sunwing's leisure network in 2025.</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
@@ -757,7 +757,7 @@
       </c>
       <c r="I6" s="3" t="inlineStr"/>
     </row>
-    <row r="7" ht="60" customHeight="1">
+    <row r="7" ht="62" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>B38M</t>
@@ -800,7 +800,7 @@
       </c>
       <c r="I7" s="5" t="inlineStr"/>
     </row>
-    <row r="8" ht="60" customHeight="1">
+    <row r="8" ht="62" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>B788</t>
@@ -847,7 +847,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="60" customHeight="1">
+    <row r="9" ht="62" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
           <t>B77W</t>
@@ -890,7 +890,7 @@
       </c>
       <c r="I9" s="5" t="inlineStr"/>
     </row>
-    <row r="10" ht="60" customHeight="1">
+    <row r="10" ht="62" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>B763</t>
@@ -933,7 +933,7 @@
       </c>
       <c r="I10" s="3" t="inlineStr"/>
     </row>
-    <row r="11" ht="60" customHeight="1">
+    <row r="11" ht="62" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
           <t>B752</t>
@@ -976,7 +976,7 @@
       </c>
       <c r="I11" s="5" t="inlineStr"/>
     </row>
-    <row r="12" ht="60" customHeight="1">
+    <row r="12" ht="62" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
           <t>E75L</t>
@@ -1019,7 +1019,7 @@
       </c>
       <c r="I12" s="3" t="inlineStr"/>
     </row>
-    <row r="13" ht="60" customHeight="1">
+    <row r="13" ht="62" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
           <t>E295</t>
@@ -1062,7 +1062,7 @@
       </c>
       <c r="I13" s="5" t="inlineStr"/>
     </row>
-    <row r="14" ht="60" customHeight="1">
+    <row r="14" ht="62" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
           <t>CRJ9</t>
@@ -1105,7 +1105,7 @@
       </c>
       <c r="I14" s="3" t="inlineStr"/>
     </row>
-    <row r="15" ht="60" customHeight="1">
+    <row r="15" ht="62" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
           <t>CRJ2</t>
@@ -1148,7 +1148,7 @@
       </c>
       <c r="I15" s="5" t="inlineStr"/>
     </row>
-    <row r="16" ht="60" customHeight="1">
+    <row r="16" ht="62" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
           <t>DH8D</t>
@@ -1195,7 +1195,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="60" customHeight="1">
+    <row r="17" ht="62" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
           <t>DH8C</t>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="I17" s="5" t="inlineStr"/>
     </row>
-    <row r="18" ht="60" customHeight="1">
+    <row r="18" ht="62" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
           <t>AT72</t>
@@ -1281,7 +1281,7 @@
       </c>
       <c r="I18" s="3" t="inlineStr"/>
     </row>
-    <row r="19" ht="60" customHeight="1">
+    <row r="19" ht="62" customHeight="1">
       <c r="A19" s="4" t="inlineStr">
         <is>
           <t>DHC6</t>
@@ -1324,7 +1324,7 @@
       </c>
       <c r="I19" s="5" t="inlineStr"/>
     </row>
-    <row r="20" ht="60" customHeight="1">
+    <row r="20" ht="62" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
           <t>C208</t>
@@ -1367,7 +1367,7 @@
       </c>
       <c r="I20" s="3" t="inlineStr"/>
     </row>
-    <row r="21" ht="60" customHeight="1">
+    <row r="21" ht="62" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
         <is>
           <t>PC12</t>
@@ -1410,7 +1410,7 @@
       </c>
       <c r="I21" s="5" t="inlineStr"/>
     </row>
-    <row r="22" ht="60" customHeight="1">
+    <row r="22" ht="62" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
           <t>C560</t>
@@ -1453,7 +1453,7 @@
       </c>
       <c r="I22" s="3" t="inlineStr"/>
     </row>
-    <row r="23" ht="60" customHeight="1">
+    <row r="23" ht="62" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
         <is>
           <t>GLEX</t>
@@ -1496,7 +1496,7 @@
       </c>
       <c r="I23" s="5" t="inlineStr"/>
     </row>
-    <row r="24" ht="60" customHeight="1">
+    <row r="24" ht="62" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
           <t>CL60</t>
@@ -1539,7 +1539,7 @@
       </c>
       <c r="I24" s="3" t="inlineStr"/>
     </row>
-    <row r="25" ht="60" customHeight="1">
+    <row r="25" ht="62" customHeight="1">
       <c r="A25" s="4" t="inlineStr">
         <is>
           <t>A310</t>
@@ -1586,7 +1586,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="60" customHeight="1">
+    <row r="26" ht="62" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
           <t>A332</t>
@@ -1633,7 +1633,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="60" customHeight="1">
+    <row r="27" ht="62" customHeight="1">
       <c r="A27" s="4" t="inlineStr">
         <is>
           <t>C130</t>
@@ -1676,7 +1676,7 @@
       </c>
       <c r="I27" s="5" t="inlineStr"/>
     </row>
-    <row r="28" ht="60" customHeight="1">
+    <row r="28" ht="62" customHeight="1">
       <c r="A28" s="2" t="inlineStr">
         <is>
           <t>C17</t>
@@ -1719,7 +1719,7 @@
       </c>
       <c r="I28" s="3" t="inlineStr"/>
     </row>
-    <row r="29" ht="60" customHeight="1">
+    <row r="29" ht="62" customHeight="1">
       <c r="A29" s="4" t="inlineStr">
         <is>
           <t>ALJT</t>
@@ -1762,7 +1762,7 @@
       </c>
       <c r="I29" s="5" t="inlineStr"/>
     </row>
-    <row r="30" ht="60" customHeight="1">
+    <row r="30" ht="62" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
           <t>F20</t>
@@ -1805,7 +1805,7 @@
       </c>
       <c r="I30" s="3" t="inlineStr"/>
     </row>
-    <row r="31" ht="60" customHeight="1">
+    <row r="31" ht="62" customHeight="1">
       <c r="A31" s="4" t="inlineStr">
         <is>
           <t>CV58</t>
@@ -1848,7 +1848,7 @@
       </c>
       <c r="I31" s="5" t="inlineStr"/>
     </row>
-    <row r="32" ht="60" customHeight="1">
+    <row r="32" ht="62" customHeight="1">
       <c r="A32" s="2" t="inlineStr">
         <is>
           <t>T-33</t>
@@ -1891,7 +1891,7 @@
       </c>
       <c r="I32" s="3" t="inlineStr"/>
     </row>
-    <row r="33" ht="60" customHeight="1">
+    <row r="33" ht="62" customHeight="1">
       <c r="A33" s="4" t="inlineStr">
         <is>
           <t>E545</t>
@@ -1934,7 +1934,7 @@
       </c>
       <c r="I33" s="5" t="inlineStr"/>
     </row>
-    <row r="34" ht="60" customHeight="1">
+    <row r="34" ht="62" customHeight="1">
       <c r="A34" s="2" t="inlineStr">
         <is>
           <t>C25B</t>
@@ -1977,7 +1977,7 @@
       </c>
       <c r="I34" s="3" t="inlineStr"/>
     </row>
-    <row r="35" ht="60" customHeight="1">
+    <row r="35" ht="62" customHeight="1">
       <c r="A35" s="4" t="inlineStr">
         <is>
           <t>LJ60</t>
@@ -2019,6 +2019,2536 @@
         </is>
       </c>
       <c r="I35" s="5" t="inlineStr"/>
+    </row>
+    <row r="36" ht="62" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>A21N</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>Airbus</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>A321neo</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>Narrowbody Jet</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>Air Canada</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>Air Canada uses long-range A321neo/XLR variants on thinner transatlantic routes, something no single-aisle jet could do economically a decade ago.</t>
+        </is>
+      </c>
+      <c r="H36" s="3" t="inlineStr">
+        <is>
+          <t>The A321XLR carries extra fuel in a permanent tank built into the rear cargo hold instead of bulky removable tanks.</t>
+        </is>
+      </c>
+      <c r="I36" s="3" t="inlineStr">
+        <is>
+          <t>"XLR" = Xtra Long Range</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="62" customHeight="1">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
+          <t>A333</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>Airbus</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>A330-300</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>Widebody Jet</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>Air Transat (seasonal)</t>
+        </is>
+      </c>
+      <c r="F37" s="5" t="inlineStr">
+        <is>
+          <t>1993</t>
+        </is>
+      </c>
+      <c r="G37" s="5" t="inlineStr">
+        <is>
+          <t>Air Transat is Canada's largest A330 operator and uses them on Ottawa's seasonal nonstop flights to Europe and sun destinations.</t>
+        </is>
+      </c>
+      <c r="H37" s="5" t="inlineStr">
+        <is>
+          <t>The A330 shares a cockpit design and type rating with the four-engine A340, so pilots can fly both with minimal extra training.</t>
+        </is>
+      </c>
+      <c r="I37" s="5" t="inlineStr"/>
+    </row>
+    <row r="38" ht="62" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>B737</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>Boeing</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>737-700</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>Narrowbody Jet</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>WestJet</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>1997</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>The 737-700 was WestJet's original workhorse when the airline launched in 1996, flying its very first routes.</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>It shares its fuselage length with the older 737-300 but uses the more modern, more efficient Next Generation wing and engines.</t>
+        </is>
+      </c>
+      <c r="I38" s="3" t="inlineStr"/>
+    </row>
+    <row r="39" ht="62" customHeight="1">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t>E190</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>Embraer</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>E190</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>Regional Jet</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>Air Canada (historic, retired 2019)</t>
+        </is>
+      </c>
+      <c r="F39" s="5" t="inlineStr">
+        <is>
+          <t>2004</t>
+        </is>
+      </c>
+      <c r="G39" s="5" t="inlineStr">
+        <is>
+          <t>Air Canada's E190s were nicknamed the "Jazz-buster" fleet internally since they let the airline fly mainline-branded service on thinner routes.</t>
+        </is>
+      </c>
+      <c r="H39" s="5" t="inlineStr">
+        <is>
+          <t>The E190 was the first regional jet with a true 2-2 seating layout and no middle seat, a first for aircraft under 100 seats.</t>
+        </is>
+      </c>
+      <c r="I39" s="5" t="inlineStr">
+        <is>
+          <t>Retired from Air Canada's fleet, but still seen visiting as charters</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="62" customHeight="1">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>CRJ7</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>Bombardier</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>CRJ700</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>Regional Jet</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>Air Canada Express (Jazz)</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>2001</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="inlineStr">
+        <is>
+          <t>The CRJ700 was stretched from the CRJ200 to add roughly 20 more seats, aimed directly at competing with Embraer's E-Jets.</t>
+        </is>
+      </c>
+      <c r="H40" s="3" t="inlineStr">
+        <is>
+          <t>It was the first Bombardier regional jet built with a supercritical wing designed specifically for the larger airframe rather than reused from the original CRJ.</t>
+        </is>
+      </c>
+      <c r="I40" s="3" t="inlineStr"/>
+    </row>
+    <row r="41" ht="62" customHeight="1">
+      <c r="A41" s="4" t="inlineStr">
+        <is>
+          <t>B77L</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>Boeing</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>777-200LR</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>Widebody Jet</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>Occasional charter/diversion</t>
+        </is>
+      </c>
+      <c r="F41" s="5" t="inlineStr">
+        <is>
+          <t>2006</t>
+        </is>
+      </c>
+      <c r="G41" s="5" t="inlineStr">
+        <is>
+          <t>The 777-200LR once set the record for the longest nonstop flight by a commercial airliner, flying Hong Kong to London the "wrong way" around the globe.</t>
+        </is>
+      </c>
+      <c r="H41" s="5" t="inlineStr">
+        <is>
+          <t>"LR" stands for Longer Range — it carries extra fuel tanks in its cargo hold like some A321 variants.</t>
+        </is>
+      </c>
+      <c r="I41" s="5" t="inlineStr">
+        <is>
+          <t>Rare visitor, usually only for special charters or diversions</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="62" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>BE35</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>Beechcraft</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>King Air 350</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>Turboprop</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>Corporate charter, air ambulance</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>1990</t>
+        </is>
+      </c>
+      <c r="G42" s="3" t="inlineStr">
+        <is>
+          <t>The King Air family is the best-selling twin-turboprop business aircraft line in history, with well over 7,000 built since 1964.</t>
+        </is>
+      </c>
+      <c r="H42" s="3" t="inlineStr">
+        <is>
+          <t>Pressurized cabins let King Airs cruise above most weather, a big reason they're a favourite for air ambulance operators across Canada.</t>
+        </is>
+      </c>
+      <c r="I42" s="3" t="inlineStr"/>
+    </row>
+    <row r="43" ht="62" customHeight="1">
+      <c r="A43" s="4" t="inlineStr">
+        <is>
+          <t>C750</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>Cessna</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>Citation X</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="inlineStr">
+        <is>
+          <t>Business Jet</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>Charter operators</t>
+        </is>
+      </c>
+      <c r="F43" s="5" t="inlineStr">
+        <is>
+          <t>1996</t>
+        </is>
+      </c>
+      <c r="G43" s="5" t="inlineStr">
+        <is>
+          <t>The Citation X was the fastest civilian aircraft in the world for years, cruising at Mach 0.92 — just a hair under the speed of sound.</t>
+        </is>
+      </c>
+      <c r="H43" s="5" t="inlineStr">
+        <is>
+          <t>Its swept wing was borrowed and adapted from fighter-jet aerodynamic research to reach that speed efficiently.</t>
+        </is>
+      </c>
+      <c r="I43" s="5" t="inlineStr"/>
+    </row>
+    <row r="44" ht="62" customHeight="1">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>C510</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>Cessna</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>Citation Mustang</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>Very Light Jet</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>Owner-operator/charter</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>2006</t>
+        </is>
+      </c>
+      <c r="G44" s="3" t="inlineStr">
+        <is>
+          <t>The Mustang helped kick off the "very light jet" category, small enough to be flown single-pilot and priced within reach of many small businesses.</t>
+        </is>
+      </c>
+      <c r="H44" s="3" t="inlineStr">
+        <is>
+          <t>It can be flown by pilots with relatively modest jet experience thanks to a simplified glass cockpit designed for owner-pilots.</t>
+        </is>
+      </c>
+      <c r="I44" s="3" t="inlineStr"/>
+    </row>
+    <row r="45" ht="62" customHeight="1">
+      <c r="A45" s="4" t="inlineStr">
+        <is>
+          <t>C680</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>Cessna</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>Citation Sovereign</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="inlineStr">
+        <is>
+          <t>Business Jet</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>Charter/corporate operators</t>
+        </is>
+      </c>
+      <c r="F45" s="5" t="inlineStr">
+        <is>
+          <t>2004</t>
+        </is>
+      </c>
+      <c r="G45" s="5" t="inlineStr">
+        <is>
+          <t>The Sovereign was designed with a wide cabin cross-section shared with Cessna's larger Citation X, giving it more headroom than most jets its size.</t>
+        </is>
+      </c>
+      <c r="H45" s="5" t="inlineStr">
+        <is>
+          <t>It's popular with corporate flight departments for its combination of a transcontinental-length cabin and short-runway capability.</t>
+        </is>
+      </c>
+      <c r="I45" s="5" t="inlineStr"/>
+    </row>
+    <row r="46" ht="62" customHeight="1">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>GLF4</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>Gulfstream</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>G450</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>Business Jet</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>Corporate/charter operators</t>
+        </is>
+      </c>
+      <c r="F46" s="3" t="inlineStr">
+        <is>
+          <t>2005</t>
+        </is>
+      </c>
+      <c r="G46" s="3" t="inlineStr">
+        <is>
+          <t>Gulfstreams are a favourite of corporate flight departments and foreign government delegations, both common visitors during Ottawa's diplomatic and parliamentary events.</t>
+        </is>
+      </c>
+      <c r="H46" s="3" t="inlineStr">
+        <is>
+          <t>The G450 can fly nonstop from Ottawa to nearly anywhere in Europe or South America without refuelling.</t>
+        </is>
+      </c>
+      <c r="I46" s="3" t="inlineStr"/>
+    </row>
+    <row r="47" ht="62" customHeight="1">
+      <c r="A47" s="4" t="inlineStr">
+        <is>
+          <t>GLF5</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>Gulfstream</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>G550</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="inlineStr">
+        <is>
+          <t>Business Jet</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>Corporate/charter, foreign government delegations</t>
+        </is>
+      </c>
+      <c r="F47" s="5" t="inlineStr">
+        <is>
+          <t>2003</t>
+        </is>
+      </c>
+      <c r="G47" s="5" t="inlineStr">
+        <is>
+          <t>The G550 has been used by NASA as a testbed and astronaut-training aircraft, alongside its usual role as a long-range executive jet.</t>
+        </is>
+      </c>
+      <c r="H47" s="5" t="inlineStr">
+        <is>
+          <t>It held multiple round-the-world and city-pair speed records after entering service.</t>
+        </is>
+      </c>
+      <c r="I47" s="5" t="inlineStr"/>
+    </row>
+    <row r="48" ht="62" customHeight="1">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>GLF6</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>Gulfstream</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>G650</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>Business Jet</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>Corporate/charter operators</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="inlineStr">
+        <is>
+          <t>2012</t>
+        </is>
+      </c>
+      <c r="G48" s="3" t="inlineStr">
+        <is>
+          <t>The G650 was, at launch, the fastest and longest-range civilian jet in the world, capable of flying from Ottawa to Tokyo nonstop.</t>
+        </is>
+      </c>
+      <c r="H48" s="3" t="inlineStr">
+        <is>
+          <t>Its cabin windows are the largest of any purpose-built business jet, nearly 40% bigger than on Gulfstream's previous models.</t>
+        </is>
+      </c>
+      <c r="I48" s="3" t="inlineStr"/>
+    </row>
+    <row r="49" ht="62" customHeight="1">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>F900</t>
+        </is>
+      </c>
+      <c r="B49" s="5" t="inlineStr">
+        <is>
+          <t>Dassault</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>Falcon 900</t>
+        </is>
+      </c>
+      <c r="D49" s="5" t="inlineStr">
+        <is>
+          <t>Business Jet</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>Corporate/charter, government delegations</t>
+        </is>
+      </c>
+      <c r="F49" s="5" t="inlineStr">
+        <is>
+          <t>1986</t>
+        </is>
+      </c>
+      <c r="G49" s="5" t="inlineStr">
+        <is>
+          <t>The Falcon 900 is one of the few business jets with three engines, a layout chosen to guarantee it could keep flying over oceans even after losing one engine.</t>
+        </is>
+      </c>
+      <c r="H49" s="5" t="inlineStr">
+        <is>
+          <t>Dassault, its manufacturer, also builds the Rafale fighter jet — Falcon business jets borrow aerodynamic know-how from that military heritage.</t>
+        </is>
+      </c>
+      <c r="I49" s="5" t="inlineStr"/>
+    </row>
+    <row r="50" ht="62" customHeight="1">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>F2TH</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>Dassault</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>Falcon 2000</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>Business Jet</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>Corporate/charter operators</t>
+        </is>
+      </c>
+      <c r="F50" s="3" t="inlineStr">
+        <is>
+          <t>1995</t>
+        </is>
+      </c>
+      <c r="G50" s="3" t="inlineStr">
+        <is>
+          <t>The Falcon 2000 was designed as a twin-engine, lower-cost complement to the tri-jet Falcon 900, sized for medium-range corporate travel.</t>
+        </is>
+      </c>
+      <c r="H50" s="3" t="inlineStr">
+        <is>
+          <t>Like all Falcons, it uses a fighter-jet-style wing designed for a smooth ride in rough air.</t>
+        </is>
+      </c>
+      <c r="I50" s="3" t="inlineStr"/>
+    </row>
+    <row r="51" ht="62" customHeight="1">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>FA7X</t>
+        </is>
+      </c>
+      <c r="B51" s="5" t="inlineStr">
+        <is>
+          <t>Dassault</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>Falcon 7X</t>
+        </is>
+      </c>
+      <c r="D51" s="5" t="inlineStr">
+        <is>
+          <t>Business Jet</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>Corporate/charter, government delegations</t>
+        </is>
+      </c>
+      <c r="F51" s="5" t="inlineStr">
+        <is>
+          <t>2007</t>
+        </is>
+      </c>
+      <c r="G51" s="5" t="inlineStr">
+        <is>
+          <t>The Falcon 7X was the first business jet with full digital fly-by-wire flight controls, technology borrowed directly from airliners and fighter jets.</t>
+        </is>
+      </c>
+      <c r="H51" s="5" t="inlineStr">
+        <is>
+          <t>It has three engines like its Falcon 900 predecessor, giving it extra range and safety margin over long ocean crossings.</t>
+        </is>
+      </c>
+      <c r="I51" s="5" t="inlineStr"/>
+    </row>
+    <row r="52" ht="62" customHeight="1">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>H25B</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>Hawker</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>800XP / 900XP</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>Business Jet</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>Charter operators</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="inlineStr">
+        <is>
+          <t>1995 (800XP)</t>
+        </is>
+      </c>
+      <c r="G52" s="3" t="inlineStr">
+        <is>
+          <t>The Hawker family traces its roots all the way back to the 1960s de Havilland DH.125, making it one of the longest continuously-produced business jet designs.</t>
+        </is>
+      </c>
+      <c r="H52" s="3" t="inlineStr">
+        <is>
+          <t>Its distinctive oval-cross-section fuselage was inherited from that 1960s design and remained largely unchanged for over 40 years of production.</t>
+        </is>
+      </c>
+      <c r="I52" s="3" t="inlineStr"/>
+    </row>
+    <row r="53" ht="62" customHeight="1">
+      <c r="A53" s="4" t="inlineStr">
+        <is>
+          <t>LJ45</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>Bombardier (Learjet)</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t>Learjet 45 / 75</t>
+        </is>
+      </c>
+      <c r="D53" s="5" t="inlineStr">
+        <is>
+          <t>Business Jet</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>Charter operators</t>
+        </is>
+      </c>
+      <c r="F53" s="5" t="inlineStr">
+        <is>
+          <t>1998</t>
+        </is>
+      </c>
+      <c r="G53" s="5" t="inlineStr">
+        <is>
+          <t>The Learjet 45 was the first all-new Learjet design in decades and the last clean-sheet Learjet before the brand's retirement in 2021.</t>
+        </is>
+      </c>
+      <c r="H53" s="5" t="inlineStr">
+        <is>
+          <t>Learjets are known for a distinctively fast, steep climb rate that pilots often describe as feeling like a fighter jet departure.</t>
+        </is>
+      </c>
+      <c r="I53" s="5" t="inlineStr"/>
+    </row>
+    <row r="54" ht="62" customHeight="1">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>PC24</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>Pilatus</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>PC-24</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>Business Jet</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>Corporate/charter operators</t>
+        </is>
+      </c>
+      <c r="F54" s="3" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="G54" s="3" t="inlineStr">
+        <is>
+          <t>The PC-24 is nicknamed the "Super Versatile Jet" because, unlike most business jets, it can operate from short, unpaved runways.</t>
+        </is>
+      </c>
+      <c r="H54" s="3" t="inlineStr">
+        <is>
+          <t>It has a large cargo door that lets it double as a light freighter or air ambulance when the cabin is reconfigured.</t>
+        </is>
+      </c>
+      <c r="I54" s="3" t="inlineStr"/>
+    </row>
+    <row r="55" ht="62" customHeight="1">
+      <c r="A55" s="4" t="inlineStr">
+        <is>
+          <t>GL7T</t>
+        </is>
+      </c>
+      <c r="B55" s="5" t="inlineStr">
+        <is>
+          <t>Bombardier</t>
+        </is>
+      </c>
+      <c r="C55" s="4" t="inlineStr">
+        <is>
+          <t>Global 7500</t>
+        </is>
+      </c>
+      <c r="D55" s="5" t="inlineStr">
+        <is>
+          <t>Business Jet</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>Corporate/charter operators</t>
+        </is>
+      </c>
+      <c r="F55" s="5" t="inlineStr">
+        <is>
+          <t>2012 (6000); 2018 (7500)</t>
+        </is>
+      </c>
+      <c r="G55" s="5" t="inlineStr">
+        <is>
+          <t>The Global 7500 can fly nonstop from Ottawa to almost any city on Earth, with a range exceeding 14,000 km.</t>
+        </is>
+      </c>
+      <c r="H55" s="5" t="inlineStr">
+        <is>
+          <t>It has four distinct living spaces in the cabin, more than any other purpose-built business jet when it launched.</t>
+        </is>
+      </c>
+      <c r="I55" s="5" t="inlineStr"/>
+    </row>
+    <row r="56" ht="62" customHeight="1">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>A139</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>Leonardo</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>AW139</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>Helicopter</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>Ornge air ambulance</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>2003</t>
+        </is>
+      </c>
+      <c r="G56" s="3" t="inlineStr">
+        <is>
+          <t>Ornge, Ontario's air ambulance service, flies AW139s in and out of The Ottawa Hospital's rooftop helipad on medevac missions around the clock.</t>
+        </is>
+      </c>
+      <c r="H56" s="3" t="inlineStr">
+        <is>
+          <t>The AW139 was co-developed by Italy's Leonardo (then Agusta) and Bell of Canada/USA before the two companies later split the program.</t>
+        </is>
+      </c>
+      <c r="I56" s="3" t="inlineStr"/>
+    </row>
+    <row r="57" ht="62" customHeight="1">
+      <c r="A57" s="4" t="inlineStr">
+        <is>
+          <t>B407</t>
+        </is>
+      </c>
+      <c r="B57" s="5" t="inlineStr">
+        <is>
+          <t>Bell</t>
+        </is>
+      </c>
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>407</t>
+        </is>
+      </c>
+      <c r="D57" s="5" t="inlineStr">
+        <is>
+          <t>Helicopter</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>Police, corporate, utility operators</t>
+        </is>
+      </c>
+      <c r="F57" s="5" t="inlineStr">
+        <is>
+          <t>1995</t>
+        </is>
+      </c>
+      <c r="G57" s="5" t="inlineStr">
+        <is>
+          <t>The Bell 407 replaced the classic Jet Ranger as the standard light helicopter for police, utility, and corporate flying across North America.</t>
+        </is>
+      </c>
+      <c r="H57" s="5" t="inlineStr">
+        <is>
+          <t>Its four-blade rotor system was adapted from Bell's OH-58D Kiowa Warrior military scout helicopter.</t>
+        </is>
+      </c>
+      <c r="I57" s="5" t="inlineStr"/>
+    </row>
+    <row r="58" ht="62" customHeight="1">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>EC35</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>Airbus Helicopters</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>H135</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>Helicopter</t>
+        </is>
+      </c>
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t>Air ambulance, corporate operators</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="inlineStr">
+        <is>
+          <t>1996</t>
+        </is>
+      </c>
+      <c r="G58" s="3" t="inlineStr">
+        <is>
+          <t>The H135's fenestron (shrouded tail rotor) makes it noticeably quieter than helicopters with a conventional exposed tail rotor — a real advantage over hospitals and neighbourhoods.</t>
+        </is>
+      </c>
+      <c r="H58" s="3" t="inlineStr">
+        <is>
+          <t>It's one of the most widely used twin-engine light helicopters for air ambulance work worldwide.</t>
+        </is>
+      </c>
+      <c r="I58" s="3" t="inlineStr"/>
+    </row>
+    <row r="59" ht="62" customHeight="1">
+      <c r="A59" s="4" t="inlineStr">
+        <is>
+          <t>C172</t>
+        </is>
+      </c>
+      <c r="B59" s="5" t="inlineStr">
+        <is>
+          <t>Cessna</t>
+        </is>
+      </c>
+      <c r="C59" s="4" t="inlineStr">
+        <is>
+          <t>172 Skyhawk</t>
+        </is>
+      </c>
+      <c r="D59" s="5" t="inlineStr">
+        <is>
+          <t>Trainer / GA</t>
+        </is>
+      </c>
+      <c r="E59" s="5" t="inlineStr">
+        <is>
+          <t>Flight schools (Ottawa Flying Club and others)</t>
+        </is>
+      </c>
+      <c r="F59" s="5" t="inlineStr">
+        <is>
+          <t>1956</t>
+        </is>
+      </c>
+      <c r="G59" s="5" t="inlineStr">
+        <is>
+          <t>The Cessna 172 is the most-produced aircraft in aviation history, with more than 44,000 built and still in production today.</t>
+        </is>
+      </c>
+      <c r="H59" s="5" t="inlineStr">
+        <is>
+          <t>It's the aircraft most private pilots in Canada, including many now flying airliners, first learned to fly on.</t>
+        </is>
+      </c>
+      <c r="I59" s="5" t="inlineStr"/>
+    </row>
+    <row r="60" ht="62" customHeight="1">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>PA28</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>Piper</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>PA-28 Cherokee / Warrior</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>Trainer / GA</t>
+        </is>
+      </c>
+      <c r="E60" s="3" t="inlineStr">
+        <is>
+          <t>Flight schools</t>
+        </is>
+      </c>
+      <c r="F60" s="3" t="inlineStr">
+        <is>
+          <t>1960</t>
+        </is>
+      </c>
+      <c r="G60" s="3" t="inlineStr">
+        <is>
+          <t>The Cherokee's simple, low-wing, single-piece-wing design made it cheaper to build and maintain than many of its rivals, helping it become a flight-school staple worldwide.</t>
+        </is>
+      </c>
+      <c r="H60" s="3" t="inlineStr">
+        <is>
+          <t>Over 90 versions of the PA-28 have been built since the 1960s, spanning trainers to fast cross-country touring aircraft.</t>
+        </is>
+      </c>
+      <c r="I60" s="3" t="inlineStr"/>
+    </row>
+    <row r="61" ht="62" customHeight="1">
+      <c r="A61" s="4" t="inlineStr">
+        <is>
+          <t>DA40</t>
+        </is>
+      </c>
+      <c r="B61" s="5" t="inlineStr">
+        <is>
+          <t>Diamond Aircraft</t>
+        </is>
+      </c>
+      <c r="C61" s="4" t="inlineStr">
+        <is>
+          <t>DA40</t>
+        </is>
+      </c>
+      <c r="D61" s="5" t="inlineStr">
+        <is>
+          <t>Trainer / GA</t>
+        </is>
+      </c>
+      <c r="E61" s="5" t="inlineStr">
+        <is>
+          <t>Flight schools</t>
+        </is>
+      </c>
+      <c r="F61" s="5" t="inlineStr">
+        <is>
+          <t>1997</t>
+        </is>
+      </c>
+      <c r="G61" s="5" t="inlineStr">
+        <is>
+          <t>Diamond's composite airframe construction (rather than traditional riveted aluminum) gives the DA40 a distinctively smooth, sleek shape for a training aircraft.</t>
+        </is>
+      </c>
+      <c r="H61" s="5" t="inlineStr">
+        <is>
+          <t>It's built in London, Ontario, making it one of relatively few aircraft you might see flying over Ottawa that's fully Canadian-built.</t>
+        </is>
+      </c>
+      <c r="I61" s="5" t="inlineStr"/>
+    </row>
+    <row r="62" ht="62" customHeight="1">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>DA42</t>
+        </is>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>Diamond Aircraft</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>DA42 Twin Star</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>Trainer / GA</t>
+        </is>
+      </c>
+      <c r="E62" s="3" t="inlineStr">
+        <is>
+          <t>Flight schools (multi-engine training)</t>
+        </is>
+      </c>
+      <c r="F62" s="3" t="inlineStr">
+        <is>
+          <t>2004</t>
+        </is>
+      </c>
+      <c r="G62" s="3" t="inlineStr">
+        <is>
+          <t>The DA42 was one of the first light twins designed from scratch around efficient diesel/Jet-A-burning engines instead of traditional avgas piston engines.</t>
+        </is>
+      </c>
+      <c r="H62" s="3" t="inlineStr">
+        <is>
+          <t>Like the DA40, it's built by Diamond Aircraft in London, Ontario.</t>
+        </is>
+      </c>
+      <c r="I62" s="3" t="inlineStr"/>
+    </row>
+    <row r="63" ht="62" customHeight="1">
+      <c r="A63" s="4" t="inlineStr">
+        <is>
+          <t>SR22</t>
+        </is>
+      </c>
+      <c r="B63" s="5" t="inlineStr">
+        <is>
+          <t>Cirrus</t>
+        </is>
+      </c>
+      <c r="C63" s="4" t="inlineStr">
+        <is>
+          <t>SR22</t>
+        </is>
+      </c>
+      <c r="D63" s="5" t="inlineStr">
+        <is>
+          <t>GA</t>
+        </is>
+      </c>
+      <c r="E63" s="5" t="inlineStr">
+        <is>
+          <t>Private owners</t>
+        </is>
+      </c>
+      <c r="F63" s="5" t="inlineStr">
+        <is>
+          <t>2001</t>
+        </is>
+      </c>
+      <c r="G63" s="5" t="inlineStr">
+        <is>
+          <t>Every Cirrus SR22 comes with a whole-airplane parachute system (CAPS) that can lower the entire aircraft safely to the ground in an emergency.</t>
+        </is>
+      </c>
+      <c r="H63" s="5" t="inlineStr">
+        <is>
+          <t>It has been the best-selling piston aircraft in the world for most years since the early 2000s.</t>
+        </is>
+      </c>
+      <c r="I63" s="5" t="inlineStr"/>
+    </row>
+    <row r="64" ht="62" customHeight="1">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>DHC2</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>De Havilland Canada</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>DHC-2 Beaver</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>Bush Plane</t>
+        </is>
+      </c>
+      <c r="E64" s="3" t="inlineStr">
+        <is>
+          <t>Occasional visitor/historic operators</t>
+        </is>
+      </c>
+      <c r="F64" s="3" t="inlineStr">
+        <is>
+          <t>1947</t>
+        </is>
+      </c>
+      <c r="G64" s="3" t="inlineStr">
+        <is>
+          <t>The Beaver was built in Toronto and is considered one of the most important Canadian aircraft ever made, engineered specifically for bush flying on floats, wheels, or skis.</t>
+        </is>
+      </c>
+      <c r="H64" s="3" t="inlineStr">
+        <is>
+          <t>The Canadian Engineering Centennial Board named the Beaver one of the top ten Canadian engineering achievements of the 20th century.</t>
+        </is>
+      </c>
+      <c r="I64" s="3" t="inlineStr">
+        <is>
+          <t>Ottawa's Canada Aviation and Space Museum, just minutes from YOW, has an original on display</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="62" customHeight="1">
+      <c r="A65" s="4" t="inlineStr">
+        <is>
+          <t>A124</t>
+        </is>
+      </c>
+      <c r="B65" s="5" t="inlineStr">
+        <is>
+          <t>Antonov</t>
+        </is>
+      </c>
+      <c r="C65" s="4" t="inlineStr">
+        <is>
+          <t>An-124 Ruslan</t>
+        </is>
+      </c>
+      <c r="D65" s="5" t="inlineStr">
+        <is>
+          <t>Heavy Cargo (rare charter)</t>
+        </is>
+      </c>
+      <c r="E65" s="5" t="inlineStr">
+        <is>
+          <t>Occasional military/oversize-cargo charters</t>
+        </is>
+      </c>
+      <c r="F65" s="5" t="inlineStr">
+        <is>
+          <t>1982</t>
+        </is>
+      </c>
+      <c r="G65" s="5" t="inlineStr">
+        <is>
+          <t>The An-124 is one of the largest cargo aircraft ever built and is sometimes chartered by the Canadian government to move outsized military or disaster-relief equipment through Ottawa.</t>
+        </is>
+      </c>
+      <c r="H65" s="5" t="inlineStr">
+        <is>
+          <t>Its cargo hold is tall and wide enough to swallow entire helicopters or armoured vehicles, loaded through a nose that swings open like a drawbridge.</t>
+        </is>
+      </c>
+      <c r="I65" s="5" t="inlineStr">
+        <is>
+          <t>A rare, unmistakable visitor when it does appear</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="62" customHeight="1">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>B744</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>Boeing</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>747-400 (Freighter)</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="inlineStr">
+        <is>
+          <t>Heavy Cargo (rare charter)</t>
+        </is>
+      </c>
+      <c r="E66" s="3" t="inlineStr">
+        <is>
+          <t>Occasional cargo charter</t>
+        </is>
+      </c>
+      <c r="F66" s="3" t="inlineStr">
+        <is>
+          <t>1989</t>
+        </is>
+      </c>
+      <c r="G66" s="3" t="inlineStr">
+        <is>
+          <t>The 747's hump-backed profile exists because Boeing originally designed the cockpit to sit above a front-loading cargo door, expecting the jet to eventually become mostly a freighter.</t>
+        </is>
+      </c>
+      <c r="H66" s="3" t="inlineStr">
+        <is>
+          <t>For over 35 years after its 1970 debut, the 747 held the title of the world's largest passenger aircraft.</t>
+        </is>
+      </c>
+      <c r="I66" s="3" t="inlineStr"/>
+    </row>
+    <row r="67" ht="62" customHeight="1">
+      <c r="A67" s="4" t="inlineStr">
+        <is>
+          <t>CH146</t>
+        </is>
+      </c>
+      <c r="B67" s="5" t="inlineStr">
+        <is>
+          <t>Bell</t>
+        </is>
+      </c>
+      <c r="C67" s="4" t="inlineStr">
+        <is>
+          <t>CH-146 Griffon</t>
+        </is>
+      </c>
+      <c r="D67" s="5" t="inlineStr">
+        <is>
+          <t>Military Helicopter</t>
+        </is>
+      </c>
+      <c r="E67" s="5" t="inlineStr">
+        <is>
+          <t>Royal Canadian Air Force (412 Transport Squadron, Ottawa)</t>
+        </is>
+      </c>
+      <c r="F67" s="5" t="inlineStr">
+        <is>
+          <t>1995</t>
+        </is>
+      </c>
+      <c r="G67" s="5" t="inlineStr">
+        <is>
+          <t>412 Transport Squadron is based right at Ottawa's airport and has flown VIP and utility helicopter support for the federal government since the 1990s.</t>
+        </is>
+      </c>
+      <c r="H67" s="5" t="inlineStr">
+        <is>
+          <t>The Griffon is a militarized version of the civilian Bell 412, itself a twin-engine development of the classic Bell 212/UH-1 "Huey" family.</t>
+        </is>
+      </c>
+      <c r="I67" s="5" t="inlineStr">
+        <is>
+          <t>Canada's most numerous military helicopter type</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="62" customHeight="1">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>B412EP</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>Bell</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>412EP</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>Helicopter</t>
+        </is>
+      </c>
+      <c r="E68" s="3" t="inlineStr">
+        <is>
+          <t>RCAF-linked and civil utility/VIP operators</t>
+        </is>
+      </c>
+      <c r="F68" s="3" t="inlineStr">
+        <is>
+          <t>1994</t>
+        </is>
+      </c>
+      <c r="G68" s="3" t="inlineStr">
+        <is>
+          <t>"EP" stands for Enhanced Performance — this variant added a better transmission and higher gross weight than the original Bell 412.</t>
+        </is>
+      </c>
+      <c r="H68" s="3" t="inlineStr">
+        <is>
+          <t>Bell 412s are built with a four-blade, soft-in-plane rotor system that gives a notably smoother ride than the two-blade Huey it descended from.</t>
+        </is>
+      </c>
+      <c r="I68" s="3" t="inlineStr"/>
+    </row>
+    <row r="69" ht="62" customHeight="1">
+      <c r="A69" s="4" t="inlineStr">
+        <is>
+          <t>B412EPI</t>
+        </is>
+      </c>
+      <c r="B69" s="5" t="inlineStr">
+        <is>
+          <t>Bell</t>
+        </is>
+      </c>
+      <c r="C69" s="4" t="inlineStr">
+        <is>
+          <t>412EPI</t>
+        </is>
+      </c>
+      <c r="D69" s="5" t="inlineStr">
+        <is>
+          <t>Helicopter</t>
+        </is>
+      </c>
+      <c r="E69" s="5" t="inlineStr">
+        <is>
+          <t>RCAF-linked and civil utility/VIP operators</t>
+        </is>
+      </c>
+      <c r="F69" s="5" t="inlineStr">
+        <is>
+          <t>2011</t>
+        </is>
+      </c>
+      <c r="G69" s="5" t="inlineStr">
+        <is>
+          <t>The 412EPI updated the Bell 412 with a modern glass cockpit, part of the same upgrade philosophy Canada later applied to extend the CH-146 Griffon's service life.</t>
+        </is>
+      </c>
+      <c r="H69" s="5" t="inlineStr">
+        <is>
+          <t>"EPI" (Enhanced Performance Improved) aircraft can often be told apart from older 412s by their flat-panel digital instrument displays visible through the windscreen.</t>
+        </is>
+      </c>
+      <c r="I69" s="5" t="inlineStr"/>
+    </row>
+    <row r="70" ht="62" customHeight="1">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>B205</t>
+        </is>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>Bell</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>205A-1++</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="inlineStr">
+        <is>
+          <t>Helicopter</t>
+        </is>
+      </c>
+      <c r="E70" s="3" t="inlineStr">
+        <is>
+          <t>Utility/forestry/fire-support operators</t>
+        </is>
+      </c>
+      <c r="F70" s="3" t="inlineStr">
+        <is>
+          <t>1971</t>
+        </is>
+      </c>
+      <c r="G70" s="3" t="inlineStr">
+        <is>
+          <t>The 205 is a civilian-certified descendant of the military UH-1 Huey, and the "++" upgrade package re-engines older airframes for hot-and-high performance decades after they were built.</t>
+        </is>
+      </c>
+      <c r="H70" s="3" t="inlineStr">
+        <is>
+          <t>Huey-family helicopters like the 205 remain popular for firefighting and heavy-lift utility work because parts and expertise are still widely available.</t>
+        </is>
+      </c>
+      <c r="I70" s="3" t="inlineStr"/>
+    </row>
+    <row r="71" ht="62" customHeight="1">
+      <c r="A71" s="4" t="inlineStr">
+        <is>
+          <t>B206</t>
+        </is>
+      </c>
+      <c r="B71" s="5" t="inlineStr">
+        <is>
+          <t>Bell</t>
+        </is>
+      </c>
+      <c r="C71" s="4" t="inlineStr">
+        <is>
+          <t>206 JetRanger / LongRanger</t>
+        </is>
+      </c>
+      <c r="D71" s="5" t="inlineStr">
+        <is>
+          <t>Helicopter</t>
+        </is>
+      </c>
+      <c r="E71" s="5" t="inlineStr">
+        <is>
+          <t>Police, tour, utility, corporate operators</t>
+        </is>
+      </c>
+      <c r="F71" s="5" t="inlineStr">
+        <is>
+          <t>1967</t>
+        </is>
+      </c>
+      <c r="G71" s="5" t="inlineStr">
+        <is>
+          <t>The Bell 206 was originally a losing entrant in a U.S. Army scout-helicopter competition — Bell reworked it into a civilian model and it went on to outsell almost every other light helicopter in history.</t>
+        </is>
+      </c>
+      <c r="H71" s="5" t="inlineStr">
+        <is>
+          <t>It's a longtime favourite for police air support, TV news, and sightseeing tours because of its low operating cost and excellent visibility bubble canopy.</t>
+        </is>
+      </c>
+      <c r="I71" s="5" t="inlineStr"/>
+    </row>
+    <row r="72" ht="62" customHeight="1">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>B429</t>
+        </is>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>Bell</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>429 GlobalRanger</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="inlineStr">
+        <is>
+          <t>Helicopter</t>
+        </is>
+      </c>
+      <c r="E72" s="3" t="inlineStr">
+        <is>
+          <t>Police, air ambulance, corporate operators</t>
+        </is>
+      </c>
+      <c r="F72" s="3" t="inlineStr">
+        <is>
+          <t>2009</t>
+        </is>
+      </c>
+      <c r="G72" s="3" t="inlineStr">
+        <is>
+          <t>The Bell 429 was the first helicopter type-certified for single-pilot IFR (instrument flight rules) operation with a full glass cockpit, letting crews fly safely at night and in poor weather.</t>
+        </is>
+      </c>
+      <c r="H72" s="3" t="inlineStr">
+        <is>
+          <t>Its distinctive four-blade rotor and twin engines make it a common choice for police air-support units and air ambulance operators across Ontario.</t>
+        </is>
+      </c>
+      <c r="I72" s="3" t="inlineStr"/>
+    </row>
+    <row r="73" ht="62" customHeight="1">
+      <c r="A73" s="4" t="inlineStr">
+        <is>
+          <t>CH47</t>
+        </is>
+      </c>
+      <c r="B73" s="5" t="inlineStr">
+        <is>
+          <t>Boeing</t>
+        </is>
+      </c>
+      <c r="C73" s="4" t="inlineStr">
+        <is>
+          <t>CH-147F Chinook</t>
+        </is>
+      </c>
+      <c r="D73" s="5" t="inlineStr">
+        <is>
+          <t>Military Helicopter</t>
+        </is>
+      </c>
+      <c r="E73" s="5" t="inlineStr">
+        <is>
+          <t>Royal Canadian Air Force (450 Tactical Helicopter Squadron)</t>
+        </is>
+      </c>
+      <c r="F73" s="5" t="inlineStr">
+        <is>
+          <t>2013 (Canadian F model)</t>
+        </is>
+      </c>
+      <c r="G73" s="5" t="inlineStr">
+        <is>
+          <t>The tandem-rotor Chinook has no tail rotor at all — its two big rotors turn in opposite directions, cancelling out the torque a normal helicopter needs a tail rotor to counter.</t>
+        </is>
+      </c>
+      <c r="H73" s="5" t="inlineStr">
+        <is>
+          <t>Canada's Chinooks are normally based in Petawawa but periodically visit Ottawa for military ceremonies, VIP support, and training moves.</t>
+        </is>
+      </c>
+      <c r="I73" s="5" t="inlineStr"/>
+    </row>
+    <row r="74" ht="62" customHeight="1">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>UH60</t>
+        </is>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>Sikorsky</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>UH-60 Black Hawk</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t>Military Helicopter</t>
+        </is>
+      </c>
+      <c r="E74" s="3" t="inlineStr">
+        <is>
+          <t>Occasional visitor — foreign military/VIP escort</t>
+        </is>
+      </c>
+      <c r="F74" s="3" t="inlineStr">
+        <is>
+          <t>1979</t>
+        </is>
+      </c>
+      <c r="G74" s="3" t="inlineStr">
+        <is>
+          <t>Canada doesn't operate Black Hawks itself, so a UH-60 over Ottawa is most often part of a visiting U.S. military detachment supporting a high-profile government or presidential visit.</t>
+        </is>
+      </c>
+      <c r="H74" s="3" t="inlineStr">
+        <is>
+          <t>The Black Hawk's airframe was designed to be survivable, with a crash-resistant structure and seats engineered to absorb impact energy in a hard landing.</t>
+        </is>
+      </c>
+      <c r="I74" s="3" t="inlineStr">
+        <is>
+          <t>A rare, notable visitor — usually tied to a specific VIP event</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="62" customHeight="1">
+      <c r="A75" s="4" t="inlineStr">
+        <is>
+          <t>AS350</t>
+        </is>
+      </c>
+      <c r="B75" s="5" t="inlineStr">
+        <is>
+          <t>Airbus Helicopters (Eurocopter)</t>
+        </is>
+      </c>
+      <c r="C75" s="4" t="inlineStr">
+        <is>
+          <t>AS350 B / "Écureuil"</t>
+        </is>
+      </c>
+      <c r="D75" s="5" t="inlineStr">
+        <is>
+          <t>Helicopter</t>
+        </is>
+      </c>
+      <c r="E75" s="5" t="inlineStr">
+        <is>
+          <t>Police, media, tour, and utility operators</t>
+        </is>
+      </c>
+      <c r="F75" s="5" t="inlineStr">
+        <is>
+          <t>1977</t>
+        </is>
+      </c>
+      <c r="G75" s="5" t="inlineStr">
+        <is>
+          <t>The AS350 ("Squirrel" in English) holds the all-time helicopter altitude landing record after one was flown to the summit of Mount Everest in 2005.</t>
+        </is>
+      </c>
+      <c r="H75" s="5" t="inlineStr">
+        <is>
+          <t>Its single Turbomeca engine and simple systems make it a favourite worldwide for police air-support, news, and aerial-survey work.</t>
+        </is>
+      </c>
+      <c r="I75" s="5" t="inlineStr"/>
+    </row>
+    <row r="76" ht="62" customHeight="1">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>DH8A</t>
+        </is>
+      </c>
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t>De Havilland Canada</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>Dash 8-100 (Flight Inspection)</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="inlineStr">
+        <is>
+          <t>Government / Calibration Aircraft</t>
+        </is>
+      </c>
+      <c r="E76" s="3" t="inlineStr">
+        <is>
+          <t>NAV CANADA</t>
+        </is>
+      </c>
+      <c r="F76" s="3" t="inlineStr">
+        <is>
+          <t>1984</t>
+        </is>
+      </c>
+      <c r="G76" s="3" t="inlineStr">
+        <is>
+          <t>NAV CANADA, the country's air navigation service provider, is headquartered in Ottawa and uses specially equipped aircraft to fly precise, repeated patterns that calibrate runway approach lights and navigation beacons at airports nationwide.</t>
+        </is>
+      </c>
+      <c r="H76" s="3" t="inlineStr">
+        <is>
+          <t>If you ever see a plane over Ottawa flying oddly repetitive loops and step-climbs, there's a good chance it's not lost — it's a flight-inspection aircraft doing its job.</t>
+        </is>
+      </c>
+      <c r="I76" s="3" t="inlineStr"/>
+    </row>
+    <row r="77" ht="62" customHeight="1">
+      <c r="A77" s="4" t="inlineStr">
+        <is>
+          <t>A359</t>
+        </is>
+      </c>
+      <c r="B77" s="5" t="inlineStr">
+        <is>
+          <t>Airbus</t>
+        </is>
+      </c>
+      <c r="C77" s="4" t="inlineStr">
+        <is>
+          <t>A350-900</t>
+        </is>
+      </c>
+      <c r="D77" s="5" t="inlineStr">
+        <is>
+          <t>Widebody Jet</t>
+        </is>
+      </c>
+      <c r="E77" s="5" t="inlineStr">
+        <is>
+          <t>Rare Air Canada visitor (maintenance ferry/diversion)</t>
+        </is>
+      </c>
+      <c r="F77" s="5" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+      <c r="G77" s="5" t="inlineStr">
+        <is>
+          <t>The A350 uses more carbon-fibre composite by weight than any other Airbus, giving it a lighter airframe and noticeably curved, downturned wingtips.</t>
+        </is>
+      </c>
+      <c r="H77" s="5" t="inlineStr">
+        <is>
+          <t>Air Canada's A350s normally fly Canada's longest routes, so spotting one over Ottawa usually means a special charter, crew-training flight, or maintenance repositioning.</t>
+        </is>
+      </c>
+      <c r="I77" s="5" t="inlineStr"/>
+    </row>
+    <row r="78" ht="62" customHeight="1">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>B739</t>
+        </is>
+      </c>
+      <c r="B78" s="3" t="inlineStr">
+        <is>
+          <t>Boeing</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>737-900ER</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="inlineStr">
+        <is>
+          <t>Narrowbody Jet</t>
+        </is>
+      </c>
+      <c r="E78" s="3" t="inlineStr">
+        <is>
+          <t>WestJet</t>
+        </is>
+      </c>
+      <c r="F78" s="3" t="inlineStr">
+        <is>
+          <t>2007</t>
+        </is>
+      </c>
+      <c r="G78" s="3" t="inlineStr">
+        <is>
+          <t>The 737-900ER is the longest version of the 737 ever built, stretched so much that it needs extra emergency exits to meet evacuation rules.</t>
+        </is>
+      </c>
+      <c r="H78" s="3" t="inlineStr">
+        <is>
+          <t>It became part of WestJet's fleet as the airline consolidated the former Sunwing leisure network into its own mainline operation in 2025.</t>
+        </is>
+      </c>
+      <c r="I78" s="3" t="inlineStr"/>
+    </row>
+    <row r="79" ht="62" customHeight="1">
+      <c r="A79" s="4" t="inlineStr">
+        <is>
+          <t>B753</t>
+        </is>
+      </c>
+      <c r="B79" s="5" t="inlineStr">
+        <is>
+          <t>Boeing</t>
+        </is>
+      </c>
+      <c r="C79" s="4" t="inlineStr">
+        <is>
+          <t>757-300</t>
+        </is>
+      </c>
+      <c r="D79" s="5" t="inlineStr">
+        <is>
+          <t>Narrowbody / Charter</t>
+        </is>
+      </c>
+      <c r="E79" s="5" t="inlineStr">
+        <is>
+          <t>Rare charter visitor</t>
+        </is>
+      </c>
+      <c r="F79" s="5" t="inlineStr">
+        <is>
+          <t>1998</t>
+        </is>
+      </c>
+      <c r="G79" s="5" t="inlineStr">
+        <is>
+          <t>The 757-300 is the longest single-aisle jet ever built by Boeing, roughly 7 metres longer than the standard 757-200.</t>
+        </is>
+      </c>
+      <c r="H79" s="5" t="inlineStr">
+        <is>
+          <t>Very few were ever built, so seeing one at Ottawa usually means a specific charter operator on a one-off flight.</t>
+        </is>
+      </c>
+      <c r="I79" s="5" t="inlineStr"/>
+    </row>
+    <row r="80" ht="62" customHeight="1">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>CN35</t>
+        </is>
+      </c>
+      <c r="B80" s="3" t="inlineStr">
+        <is>
+          <t>Canadian North</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>737-300 Combi</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="inlineStr">
+        <is>
+          <t>Narrowbody / Passenger-Cargo Combi</t>
+        </is>
+      </c>
+      <c r="E80" s="3" t="inlineStr">
+        <is>
+          <t>Canadian North</t>
+        </is>
+      </c>
+      <c r="F80" s="3" t="inlineStr">
+        <is>
+          <t>1985 (737-300)</t>
+        </is>
+      </c>
+      <c r="G80" s="3" t="inlineStr">
+        <is>
+          <t>A "Combi" jet carries cargo pallets in the front of the cabin and passengers in the back behind a partition — a practical setup for flying both people and freight to Canada's North.</t>
+        </is>
+      </c>
+      <c r="H80" s="3" t="inlineStr">
+        <is>
+          <t>Canadian North was formed by merging two historic northern carriers, First Air and Canadian North, in 2019.</t>
+        </is>
+      </c>
+      <c r="I80" s="3" t="inlineStr"/>
+    </row>
+    <row r="81" ht="62" customHeight="1">
+      <c r="A81" s="4" t="inlineStr">
+        <is>
+          <t>SW4</t>
+        </is>
+      </c>
+      <c r="B81" s="5" t="inlineStr">
+        <is>
+          <t>Fairchild (Swearingen)</t>
+        </is>
+      </c>
+      <c r="C81" s="4" t="inlineStr">
+        <is>
+          <t>Metro/Merlin III</t>
+        </is>
+      </c>
+      <c r="D81" s="5" t="inlineStr">
+        <is>
+          <t>Turboprop / Small Freighter</t>
+        </is>
+      </c>
+      <c r="E81" s="5" t="inlineStr">
+        <is>
+          <t>Small feeder-cargo operators</t>
+        </is>
+      </c>
+      <c r="F81" s="5" t="inlineStr">
+        <is>
+          <t>1970</t>
+        </is>
+      </c>
+      <c r="G81" s="5" t="inlineStr">
+        <is>
+          <t>The Metroliner's narrow, cylindrical fuselage earned it the nickname "the Lead Sled" among pilots for its dense, no-nonsense build.</t>
+        </is>
+      </c>
+      <c r="H81" s="5" t="inlineStr">
+        <is>
+          <t>Small Metros have flown overnight parcel and bank-cheque runs into Ottawa for decades, often departing in the middle of the night.</t>
+        </is>
+      </c>
+      <c r="I81" s="5" t="inlineStr">
+        <is>
+          <t>Nickname: "Lead Sled"</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="62" customHeight="1">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>GL5T</t>
+        </is>
+      </c>
+      <c r="B82" s="3" t="inlineStr">
+        <is>
+          <t>Bombardier</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>Global 5000</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="inlineStr">
+        <is>
+          <t>Business Jet</t>
+        </is>
+      </c>
+      <c r="E82" s="3" t="inlineStr">
+        <is>
+          <t>Corporate/charter operators</t>
+        </is>
+      </c>
+      <c r="F82" s="3" t="inlineStr">
+        <is>
+          <t>2005</t>
+        </is>
+      </c>
+      <c r="G82" s="3" t="inlineStr">
+        <is>
+          <t>The Global 5000 was developed alongside the Global Express as a shorter-range, lower-cost sibling, sharing most of the same wing and cockpit.</t>
+        </is>
+      </c>
+      <c r="H82" s="3" t="inlineStr">
+        <is>
+          <t>It's a common choice for corporate flight departments needing nonstop Ottawa-to-Europe range without paying for the largest Global variant.</t>
+        </is>
+      </c>
+      <c r="I82" s="3" t="inlineStr"/>
+    </row>
+    <row r="83" ht="62" customHeight="1">
+      <c r="A83" s="4" t="inlineStr">
+        <is>
+          <t>E55P</t>
+        </is>
+      </c>
+      <c r="B83" s="5" t="inlineStr">
+        <is>
+          <t>Embraer</t>
+        </is>
+      </c>
+      <c r="C83" s="4" t="inlineStr">
+        <is>
+          <t>Praetor 600</t>
+        </is>
+      </c>
+      <c r="D83" s="5" t="inlineStr">
+        <is>
+          <t>Business Jet</t>
+        </is>
+      </c>
+      <c r="E83" s="5" t="inlineStr">
+        <is>
+          <t>Corporate/charter operators</t>
+        </is>
+      </c>
+      <c r="F83" s="5" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="G83" s="5" t="inlineStr">
+        <is>
+          <t>The Praetor 600 was the first mid-size business jet certified for "fly-by-wire" flight controls, technology normally reserved for larger jets.</t>
+        </is>
+      </c>
+      <c r="H83" s="5" t="inlineStr">
+        <is>
+          <t>Embraer says its cabin altitude (effectively how much oxygen you feel at cruise) is among the lowest of any business jet in its class, reducing jet-lag fatigue.</t>
+        </is>
+      </c>
+      <c r="I83" s="5" t="inlineStr"/>
+    </row>
+    <row r="84" ht="62" customHeight="1">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>C68A</t>
+        </is>
+      </c>
+      <c r="B84" s="3" t="inlineStr">
+        <is>
+          <t>Cessna</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>Citation Latitude</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="inlineStr">
+        <is>
+          <t>Business Jet</t>
+        </is>
+      </c>
+      <c r="E84" s="3" t="inlineStr">
+        <is>
+          <t>Corporate/charter operators</t>
+        </is>
+      </c>
+      <c r="F84" s="3" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+      <c r="G84" s="3" t="inlineStr">
+        <is>
+          <t>The Latitude has a flat cabin floor, unusual for a mid-size jet, making it feel noticeably roomier inside than its exterior size suggests.</t>
+        </is>
+      </c>
+      <c r="H84" s="3" t="inlineStr">
+        <is>
+          <t>It quickly became one of Cessna's best-selling business jets after launch thanks to its combination of cabin comfort and short-runway capability.</t>
+        </is>
+      </c>
+      <c r="I84" s="3" t="inlineStr"/>
+    </row>
+    <row r="85" ht="62" customHeight="1">
+      <c r="A85" s="4" t="inlineStr">
+        <is>
+          <t>PRM1</t>
+        </is>
+      </c>
+      <c r="B85" s="5" t="inlineStr">
+        <is>
+          <t>Beechcraft</t>
+        </is>
+      </c>
+      <c r="C85" s="4" t="inlineStr">
+        <is>
+          <t>Premier 1</t>
+        </is>
+      </c>
+      <c r="D85" s="5" t="inlineStr">
+        <is>
+          <t>Business Jet</t>
+        </is>
+      </c>
+      <c r="E85" s="5" t="inlineStr">
+        <is>
+          <t>Owner-operator/charter</t>
+        </is>
+      </c>
+      <c r="F85" s="5" t="inlineStr">
+        <is>
+          <t>2001</t>
+        </is>
+      </c>
+      <c r="G85" s="5" t="inlineStr">
+        <is>
+          <t>The Premier 1 was one of the first business jets with a composite-material fuselage, built as a single-piece carbon-fibre barrel instead of riveted aluminum panels.</t>
+        </is>
+      </c>
+      <c r="H85" s="5" t="inlineStr">
+        <is>
+          <t>It's designed to be flown single-pilot, keeping operating costs down for private owners.</t>
+        </is>
+      </c>
+      <c r="I85" s="5" t="inlineStr"/>
+    </row>
+    <row r="86" ht="62" customHeight="1">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>PA34</t>
+        </is>
+      </c>
+      <c r="B86" s="3" t="inlineStr">
+        <is>
+          <t>Piper</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>PA-34 Seneca</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="inlineStr">
+        <is>
+          <t>Trainer / GA (multi-engine)</t>
+        </is>
+      </c>
+      <c r="E86" s="3" t="inlineStr">
+        <is>
+          <t>Flight schools</t>
+        </is>
+      </c>
+      <c r="F86" s="3" t="inlineStr">
+        <is>
+          <t>1971</t>
+        </is>
+      </c>
+      <c r="G86" s="3" t="inlineStr">
+        <is>
+          <t>The Seneca is one of the most common aircraft Canadian pilots use to earn their multi-engine rating, the qualification needed to fly twin-engine aircraft.</t>
+        </is>
+      </c>
+      <c r="H86" s="3" t="inlineStr">
+        <is>
+          <t>Its two engines are mounted close to the fuselage centerline, which makes it noticeably easier to control on one engine than many other light twins.</t>
+        </is>
+      </c>
+      <c r="I86" s="3" t="inlineStr"/>
+    </row>
+    <row r="87" ht="62" customHeight="1">
+      <c r="A87" s="4" t="inlineStr">
+        <is>
+          <t>BE36</t>
+        </is>
+      </c>
+      <c r="B87" s="5" t="inlineStr">
+        <is>
+          <t>Beechcraft</t>
+        </is>
+      </c>
+      <c r="C87" s="4" t="inlineStr">
+        <is>
+          <t>Bonanza</t>
+        </is>
+      </c>
+      <c r="D87" s="5" t="inlineStr">
+        <is>
+          <t>GA</t>
+        </is>
+      </c>
+      <c r="E87" s="5" t="inlineStr">
+        <is>
+          <t>Private owners</t>
+        </is>
+      </c>
+      <c r="F87" s="5" t="inlineStr">
+        <is>
+          <t>1947</t>
+        </is>
+      </c>
+      <c r="G87" s="5" t="inlineStr">
+        <is>
+          <t>The Bonanza has been in continuous production longer than any other airplane in history, with the same basic design still being built today.</t>
+        </is>
+      </c>
+      <c r="H87" s="5" t="inlineStr">
+        <is>
+          <t>Early models had a distinctive V-shaped tail (the "V-tail Bonanza") that combined the rudder and elevator into just two control surfaces instead of three.</t>
+        </is>
+      </c>
+      <c r="I87" s="5" t="inlineStr"/>
+    </row>
+    <row r="88" ht="62" customHeight="1">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>RV_</t>
+        </is>
+      </c>
+      <c r="B88" s="3" t="inlineStr">
+        <is>
+          <t>Van's Aircraft</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>RV Series</t>
+        </is>
+      </c>
+      <c r="D88" s="3" t="inlineStr">
+        <is>
+          <t>Homebuilt / GA</t>
+        </is>
+      </c>
+      <c r="E88" s="3" t="inlineStr">
+        <is>
+          <t>Private owners (based at Rockcliffe, Carp, and other local airfields)</t>
+        </is>
+      </c>
+      <c r="F88" s="3" t="inlineStr">
+        <is>
+          <t>1972</t>
+        </is>
+      </c>
+      <c r="G88" s="3" t="inlineStr">
+        <is>
+          <t>Van's RV kits are the best-selling homebuilt aircraft design in the world — owners assemble them themselves, often over several years in a home garage.</t>
+        </is>
+      </c>
+      <c r="H88" s="3" t="inlineStr">
+        <is>
+          <t>Despite being amateur-built, RVs are known for genuinely sporty, responsive handling that rivals purpose-built aerobatic aircraft.</t>
+        </is>
+      </c>
+      <c r="I88" s="3" t="inlineStr"/>
+    </row>
+    <row r="89" ht="62" customHeight="1">
+      <c r="A89" s="4" t="inlineStr">
+        <is>
+          <t>VC25</t>
+        </is>
+      </c>
+      <c r="B89" s="5" t="inlineStr">
+        <is>
+          <t>Boeing</t>
+        </is>
+      </c>
+      <c r="C89" s="4" t="inlineStr">
+        <is>
+          <t>VC-25 (Air Force One)</t>
+        </is>
+      </c>
+      <c r="D89" s="5" t="inlineStr">
+        <is>
+          <t>Government / Head-of-State Transport</t>
+        </is>
+      </c>
+      <c r="E89" s="5" t="inlineStr">
+        <is>
+          <t>Extremely rare — U.S. presidential visits only</t>
+        </is>
+      </c>
+      <c r="F89" s="5" t="inlineStr">
+        <is>
+          <t>1990</t>
+        </is>
+      </c>
+      <c r="G89" s="5" t="inlineStr">
+        <is>
+          <t>"Air Force One" isn't really an aircraft type — it's the call sign used by any U.S. Air Force aircraft carrying the President, though it almost always refers to the specially modified 747 VC-25.</t>
+        </is>
+      </c>
+      <c r="H89" s="5" t="inlineStr">
+        <is>
+          <t>The VC-25 can be refuelled in mid-air, giving it, in theory, unlimited range for as long as the crew can stay awake.</t>
+        </is>
+      </c>
+      <c r="I89" s="5" t="inlineStr">
+        <is>
+          <t>One of the rarest possible sightings at YOW — only during an official presidential visit</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="62" customHeight="1">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>C32</t>
+        </is>
+      </c>
+      <c r="B90" s="3" t="inlineStr">
+        <is>
+          <t>Boeing</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>C-32 (757)</t>
+        </is>
+      </c>
+      <c r="D90" s="3" t="inlineStr">
+        <is>
+          <t>Government / VIP Transport</t>
+        </is>
+      </c>
+      <c r="E90" s="3" t="inlineStr">
+        <is>
+          <t>Rare — U.S. government/VIP visits</t>
+        </is>
+      </c>
+      <c r="F90" s="3" t="inlineStr">
+        <is>
+          <t>1998</t>
+        </is>
+      </c>
+      <c r="G90" s="3" t="inlineStr">
+        <is>
+          <t>The C-32 is a militarized 757 used by the U.S. Air Force to fly the Vice President, First Lady, Secretary of State, and other senior officials — commonly seen supporting high-level visits to Ottawa.</t>
+        </is>
+      </c>
+      <c r="H90" s="3" t="inlineStr">
+        <is>
+          <t>It carries advanced communications equipment so senior officials can stay in contact with Washington throughout the flight.</t>
+        </is>
+      </c>
+      <c r="I90" s="3" t="inlineStr"/>
+    </row>
+    <row r="91" ht="62" customHeight="1">
+      <c r="A91" s="4" t="inlineStr">
+        <is>
+          <t>C5M</t>
+        </is>
+      </c>
+      <c r="B91" s="5" t="inlineStr">
+        <is>
+          <t>Lockheed Martin</t>
+        </is>
+      </c>
+      <c r="C91" s="4" t="inlineStr">
+        <is>
+          <t>C-5M Super Galaxy</t>
+        </is>
+      </c>
+      <c r="D91" s="5" t="inlineStr">
+        <is>
+          <t>Military Transport</t>
+        </is>
+      </c>
+      <c r="E91" s="5" t="inlineStr">
+        <is>
+          <t>Rare — U.S. heavy-airlift support</t>
+        </is>
+      </c>
+      <c r="F91" s="5" t="inlineStr">
+        <is>
+          <t>1969 (C-5); 2013 (M upgrade)</t>
+        </is>
+      </c>
+      <c r="G91" s="5" t="inlineStr">
+        <is>
+          <t>The C-5 is one of the largest military aircraft in the world — its cargo hold is long enough to fit multiple helicopters or armoured vehicles nose to tail.</t>
+        </is>
+      </c>
+      <c r="H91" s="5" t="inlineStr">
+        <is>
+          <t>Both the nose and tail of the aircraft open, letting crews drive vehicles straight through from one end to the other.</t>
+        </is>
+      </c>
+      <c r="I91" s="5" t="inlineStr"/>
+    </row>
+    <row r="92" ht="62" customHeight="1">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>K35R</t>
+        </is>
+      </c>
+      <c r="B92" s="3" t="inlineStr">
+        <is>
+          <t>Boeing</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>KC-135 Stratotanker</t>
+        </is>
+      </c>
+      <c r="D92" s="3" t="inlineStr">
+        <is>
+          <t>Military Tanker</t>
+        </is>
+      </c>
+      <c r="E92" s="3" t="inlineStr">
+        <is>
+          <t>Rare — U.S. escort/support aircraft</t>
+        </is>
+      </c>
+      <c r="F92" s="3" t="inlineStr">
+        <is>
+          <t>1957</t>
+        </is>
+      </c>
+      <c r="G92" s="3" t="inlineStr">
+        <is>
+          <t>The KC-135 shares its basic airframe design with the original Boeing 707 airliner and has remained in continuous U.S. Air Force service for well over 60 years.</t>
+        </is>
+      </c>
+      <c r="H92" s="3" t="inlineStr">
+        <is>
+          <t>It refuels other aircraft in flight through a rigid, steerable "flying boom" operated by a crew member lying in the tail of the plane.</t>
+        </is>
+      </c>
+      <c r="I92" s="3" t="inlineStr"/>
+    </row>
+    <row r="93" ht="62" customHeight="1">
+      <c r="A93" s="4" t="inlineStr">
+        <is>
+          <t>C40</t>
+        </is>
+      </c>
+      <c r="B93" s="5" t="inlineStr">
+        <is>
+          <t>Boeing</t>
+        </is>
+      </c>
+      <c r="C93" s="4" t="inlineStr">
+        <is>
+          <t>C-40 Clipper</t>
+        </is>
+      </c>
+      <c r="D93" s="5" t="inlineStr">
+        <is>
+          <t>Government / VIP Transport</t>
+        </is>
+      </c>
+      <c r="E93" s="5" t="inlineStr">
+        <is>
+          <t>Rare — U.S. military/VIP visits</t>
+        </is>
+      </c>
+      <c r="F93" s="5" t="inlineStr">
+        <is>
+          <t>2001</t>
+        </is>
+      </c>
+      <c r="G93" s="5" t="inlineStr">
+        <is>
+          <t>The C-40 is a militarized Boeing 737-700 used by the U.S. Navy, Air Force, and Air National Guard to fly senior officials and congressional delegations.</t>
+        </is>
+      </c>
+      <c r="H93" s="5" t="inlineStr">
+        <is>
+          <t>It's built on the same production line as Boeing's commercial 737 Next Generation jets, just with a stronger cargo floor and VIP interior.</t>
+        </is>
+      </c>
+      <c r="I93" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>